<commit_message>
chore : update excel example for transaksi spp/bpp
</commit_message>
<xml_diff>
--- a/public/assets/files/Contoh Format Import Flow Pembayaran Bulanan.xlsx
+++ b/public/assets/files/Contoh Format Import Flow Pembayaran Bulanan.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\xampp_8.1.6\htdocs\illiyin\sikas\public\assets\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wazirul\Documents\Sikas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6EE98D1-47CB-48C6-B195-587D045A0281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAB1DDA-2405-4838-92F0-68686660F5D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Contoh Format Bulanan" sheetId="6" r:id="rId1"/>
+    <sheet name="TKJ" sheetId="6" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="66">
   <si>
     <t>Nama</t>
   </si>
@@ -81,24 +81,9 @@
     <t xml:space="preserve"> yaitu Aktif (Siswa yang masih aktif bersekolah) dan Alumni (Siswa yang sudah tidak bersekolah / lulus)</t>
   </si>
   <si>
-    <t>5. Sisa Partisipasi adalah sisa tanggungan siswa untuk membayar spp/bpp</t>
-  </si>
-  <si>
     <t>1. Sebelum mengimport Data Pembayaran BPP, pastikan Data Siswa sudah di IMPORT sebelumnya</t>
   </si>
   <si>
-    <t>2. Jenis Kelamin terdiri dari L (Laki-Laki) &amp; P (Perempuan)</t>
-  </si>
-  <si>
-    <t>3. Status Siswa terdiri dari 2 status,</t>
-  </si>
-  <si>
-    <t>4. Pastikan Jurusan siswa yang akan di import sudah dibuat oleh Admin.</t>
-  </si>
-  <si>
-    <t>6. Total Bayar adalah total pembayaran siswa dalam membayar spp/bpp</t>
-  </si>
-  <si>
     <t>No. Induk</t>
   </si>
   <si>
@@ -108,18 +93,9 @@
     <t>XI-TKJ-2</t>
   </si>
   <si>
-    <t>7. Flow Pembayaran terdiri dari 2 flow yaitu Angsuran &amp; Bulanan</t>
-  </si>
-  <si>
-    <t>8. Angkatan Tahun adalah kolom itu siswa lulus tahun berapa / alumni lulus tahun berapa</t>
-  </si>
-  <si>
     <t>Flow Pembayaran</t>
   </si>
   <si>
-    <t>Angkatan Tahun</t>
-  </si>
-  <si>
     <t>Bulanan</t>
   </si>
   <si>
@@ -168,9 +144,6 @@
     <t>Total Kesanggupan Pertahun</t>
   </si>
   <si>
-    <t>9. Total Kesanggupan Pertahun harus diisi sesuai nominalnya</t>
-  </si>
-  <si>
     <t>10. Pembayaran Angsuran harus diisi dengan nominal angka, jangan teks / kata2</t>
   </si>
   <si>
@@ -208,6 +181,54 @@
   </si>
   <si>
     <t>Alumni</t>
+  </si>
+  <si>
+    <t>2021-2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2. Jangan merubah susunan kolom yang telah disediakan</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> susunan excel harus sama sesuai dengan format yang telah disediakan</t>
+  </si>
+  <si>
+    <t>3. Jenis Kelamin terdiri dari L (Laki-Laki) &amp; P (Perempuan)</t>
+  </si>
+  <si>
+    <t>4. Status Siswa terdiri dari 2 status,</t>
+  </si>
+  <si>
+    <t>5. Pastikan Jurusan siswa yang akan di import sudah dibuat oleh Admin.</t>
+  </si>
+  <si>
+    <t>6. Flow Pembayaran terdiri dari 2 flow yaitu Angsuran &amp; Bulanan</t>
+  </si>
+  <si>
+    <t>7. Tahun Ajaran digunakan untuk mengisi tahun ajaran siswa tersebut</t>
+  </si>
+  <si>
+    <t>8. Angkatan Tahun adalah kolom yang digunakan untuk tahun siswa tersebut lulus</t>
+  </si>
+  <si>
+    <t>9. Total Kesanggupan Pertahun harus diisi sesuai nominalnya, sesuai dengan kesanggupan siswa,</t>
+  </si>
+  <si>
+    <t>11. Sisa Partisipasi adalah sisa tanggungan siswa untuk membayar spp/bpp</t>
+  </si>
+  <si>
+    <t>12. Total Bayar adalah total pembayaran siswa dalam membayar spp/bpp</t>
+  </si>
+  <si>
+    <t>13. Tidak perlu mengisi kelebihan dan kekurangan tahun sebelumnya jika data import tahun ajar lengkap</t>
+  </si>
+  <si>
+    <t>Tahun Ajaran</t>
+  </si>
+  <si>
+    <t>Angkatan Tahun (Alumni)</t>
+  </si>
+  <si>
+    <t>2022-2023</t>
   </si>
 </sst>
 </file>
@@ -217,11 +238,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-[$Rp-421]* #,##0_-;\-[$Rp-421]* #,##0_-;_-[$Rp-421]* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -281,6 +309,20 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -346,48 +388,53 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E36714-8EFC-4E0B-B83E-061AD658FD81}">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AB19"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.33203125" customWidth="1"/>
@@ -619,19 +666,19 @@
     <col min="4" max="4" width="22.109375" customWidth="1"/>
     <col min="5" max="5" width="18.109375" customWidth="1"/>
     <col min="6" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="8" width="22.44140625" customWidth="1"/>
-    <col min="9" max="11" width="22.109375" customWidth="1"/>
-    <col min="12" max="23" width="12.21875" customWidth="1"/>
-    <col min="24" max="25" width="22.109375" customWidth="1"/>
-    <col min="27" max="27" width="90.88671875" style="9" customWidth="1"/>
+    <col min="7" max="9" width="22.44140625" customWidth="1"/>
+    <col min="10" max="12" width="22.109375" customWidth="1"/>
+    <col min="13" max="24" width="12.21875" customWidth="1"/>
+    <col min="25" max="26" width="22.109375" customWidth="1"/>
+    <col min="28" max="28" width="101.44140625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -646,315 +693,359 @@
         <v>2</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="T1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="4">
+        <v>600000</v>
+      </c>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7">
+        <v>100000</v>
+      </c>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7">
+        <v>200000</v>
+      </c>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7">
+        <v>300000</v>
+      </c>
+      <c r="Z2" s="7">
+        <v>300000</v>
+      </c>
+      <c r="AB2" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="4">
+        <v>600000</v>
+      </c>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="7">
+        <v>600000</v>
+      </c>
+      <c r="Z3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="4">
+        <v>600000</v>
+      </c>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="7"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="7">
+        <v>600000</v>
+      </c>
+      <c r="Z4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="S1" s="2" t="s">
+      <c r="D5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="4">
+        <v>600000</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="7">
+        <v>600000</v>
+      </c>
+      <c r="Z5" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB6" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB7" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB8" s="13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB9" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB10" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB11" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB12" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB13" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" s="5">
-        <v>600000</v>
-      </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8">
-        <v>100000</v>
-      </c>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8">
-        <v>200000</v>
-      </c>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
-      <c r="U2" s="8"/>
-      <c r="V2" s="8"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8">
-        <v>300000</v>
-      </c>
-      <c r="Y2" s="8">
-        <v>300000</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="5">
-        <v>600000</v>
-      </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8"/>
-      <c r="S3" s="8"/>
-      <c r="T3" s="8"/>
-      <c r="U3" s="8"/>
-      <c r="V3" s="8"/>
-      <c r="W3" s="8"/>
-      <c r="X3" s="8">
-        <v>600000</v>
-      </c>
-      <c r="Y3" s="8">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="5">
-        <v>600000</v>
-      </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8"/>
-      <c r="S4" s="8"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="8"/>
-      <c r="V4" s="8"/>
-      <c r="W4" s="8"/>
-      <c r="X4" s="8">
-        <v>600000</v>
-      </c>
-      <c r="Y4" s="8">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="5">
-        <v>600000</v>
-      </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="8"/>
-      <c r="W5" s="8"/>
-      <c r="X5" s="8">
-        <v>600000</v>
-      </c>
-      <c r="Y5" s="8">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA6" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA7" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA8" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA9" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA10" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA11" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA12" s="3" t="s">
-        <v>46</v>
-      </c>
+    </row>
+    <row r="14" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB14" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB15" s="13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="AB16" s="13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" spans="28:28" ht="15" x14ac:dyDescent="0.25">
+      <c r="AB17" s="16"/>
+    </row>
+    <row r="18" spans="28:28" ht="15" x14ac:dyDescent="0.25">
+      <c r="AB18" s="16"/>
+    </row>
+    <row r="19" spans="28:28" ht="15" x14ac:dyDescent="0.25">
+      <c r="AB19" s="16"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>